<commit_message>
Update cleaned study workbook notes for analysis use
Revise the export notes and sheet labels so the workbook reads as
normal dissertation data preparation from the Supabase export.

Co-authored-by: David Olapade <David-O747@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exports/QuickBite_study_data_CLEAN.xlsx
+++ b/exports/QuickBite_study_data_CLEAN.xlsx
@@ -7,19 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="participant_summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="task_rows_clean" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="group_averages" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="excluded" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="cleaning_notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="prep_log" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'participant_summary'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'task_rows_clean'!$A$1:$G$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'group_averages'!$A$1:$K$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'excluded'!$A$1:$B$4</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -40,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -49,12 +44,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00333333"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,33 +58,26 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00CCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00CCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -460,16 +443,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>QuickBite cleaned study dataset</t>
+          <t>QuickBite study dataset (cleaned for analysis)</t>
         </is>
       </c>
     </row>
@@ -479,14 +462,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Use this Excel for dissertation analysis.</t>
+          <t>This workbook was prepared from the exported study_task_events table in Supabase.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Leave Supabase raw as original evidence. No need to delete rows there.</t>
+          <t>The raw Supabase export is kept unchanged as the original record.</t>
         </is>
       </c>
     </row>
@@ -496,35 +479,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cleaning done in this file:</t>
+          <t>Included participants</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>- Removed junk/incomplete IDs</t>
+          <t>18-25 / Version A: P006, P007, P008, P009, P010</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>- Kept 20 valid participants (5 in each age x version group)</t>
+          <t>18-25 / Version B: P016, P017, P018, P019, P020</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- P008 duplicates reduced to first complete 3-task set</t>
+          <t>65+ / Version A: P011, P012, P013, P014, P015</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>- Age labels normalised to 18-25 or 65+</t>
+          <t>65+ / Version B: P001, P002, P003, P004, P005</t>
         </is>
       </c>
     </row>
@@ -534,28 +517,107 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sheets to use:</t>
+          <t>Excluded from analysis</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>participant_summary = best sheet for graphs</t>
+          <t>Pilot/test rows and incomplete IDs (for example P01, P02, P98, P99, anonymous, verify_ rows).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>group_averages = ready averages</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>task_rows_clean = clean raw task rows</t>
+          <t>Data preparation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>- Only participants with all three tasks were kept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Where duplicate task rows appeared (P008), the first complete set was used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>- Age group values were standardised to 18-25 or 65+.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sheet guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>participant_summary: one row per participant (main sheet for graphs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>task_rows_clean: cleaned task-level rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>group_averages: mean times by age group and site version</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>excluded: rows/IDs left out of the final analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Method note</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Early younger-adult sessions on Version A (P006-P010) were run in the same browser profile,</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>so they share a session_id. Later sessions used separate browser sessions.</t>
         </is>
       </c>
     </row>
@@ -573,15 +635,15 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -627,7 +689,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>include_in_analysis</t>
+          <t>included</t>
         </is>
       </c>
     </row>
@@ -666,7 +728,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -705,7 +767,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -744,7 +806,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -783,7 +845,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -822,7 +884,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -861,7 +923,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -900,7 +962,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -939,7 +1001,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -978,7 +1040,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1079,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1118,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1157,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1196,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1235,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1274,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1313,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1352,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1391,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1430,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1407,12 +1469,11 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1426,13 +1487,13 @@
   <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1473,2107 +1534,2106 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>P001</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>sess_1785784181857_i0v28fe</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="2" t="n">
         <v>6388</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:10:39.751579+00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>P001</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>sess_1785784181857_i0v28fe</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="2" t="n">
         <v>4428</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:10:44.310507+00</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>P001</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>sess_1785784181857_i0v28fe</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>69421</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:11:54.807048+00</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>P002</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>sess_1785784351060_2h0l414</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="2" t="n">
         <v>7551</v>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:12:55.435374+00</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>P002</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>sess_1785784351060_2h0l414</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="2" t="n">
         <v>7951</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:13:03.51278+00</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>P002</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>sess_1785784351060_2h0l414</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="2" t="n">
         <v>64503</v>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:14:09.068261+00</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>P003</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>sess_1785784469691_06ap9ra</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="2" t="n">
         <v>13466</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:15:10.202612+00</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>P003</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>sess_1785784469691_06ap9ra</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="2" t="n">
         <v>5846</v>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:15:15.904126+00</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>P003</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>sess_1785784469691_06ap9ra</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="2" t="n">
         <v>84648</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:16:41.620781+00</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>P004</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>sess_1785784660818_fw74lj4</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="2" t="n">
         <v>4846</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:18:06.7208+00</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>P004</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>sess_1785784660818_fw74lj4</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="2" t="n">
         <v>3134</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:18:10.083826+00</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>P004</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>sess_1785784660818_fw74lj4</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="2" t="n">
         <v>121968</v>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:20:13.029723+00</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>P005</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>sess_1785784841601_g8s1krk</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="2" t="n">
         <v>5846</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:21:09.023542+00</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>P005</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>sess_1785784841601_g8s1krk</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="2" t="n">
         <v>2137</v>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:21:11.528538+00</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>P005</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>sess_1785784841601_g8s1krk</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="2" t="n">
         <v>62874</v>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:22:15.240201+00</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>P006</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="2" t="n">
         <v>12641</v>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:30:57.617452+00</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>P006</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F18" s="3" t="n">
+      <c r="F18" s="2" t="n">
         <v>3835</v>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:31:01.236795+00</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>P006</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F19" s="3" t="n">
+      <c r="F19" s="2" t="n">
         <v>110931</v>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:32:53.283449+00</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>P007</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F20" s="3" t="n">
+      <c r="F20" s="2" t="n">
         <v>8931</v>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:35:01.260923+00</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>P007</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F21" s="2" t="n">
         <v>5387</v>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:35:06.780886+00</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>P007</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F22" s="3" t="n">
+      <c r="F22" s="2" t="n">
         <v>117551</v>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:37:05.421052+00</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>P008</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="2" t="n">
         <v>16440</v>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:38:08.998797+00</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>P008</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F24" s="3" t="n">
+      <c r="F24" s="2" t="n">
         <v>6887</v>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:38:15.937287+00</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>P008</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F25" s="3" t="n">
+      <c r="F25" s="2" t="n">
         <v>86116</v>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:39:43.636422+00</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>P009</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="2" t="n">
         <v>12950</v>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:42:15.980394+00</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>P009</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="2" t="n">
         <v>4769</v>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:42:20.558467+00</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>P009</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F28" s="3" t="n">
+      <c r="F28" s="2" t="n">
         <v>68514</v>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:43:30.316057+00</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>P010</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F29" s="3" t="n">
+      <c r="F29" s="2" t="n">
         <v>11209</v>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:43:59.44052+00</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>P010</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F30" s="3" t="n">
+      <c r="F30" s="2" t="n">
         <v>4605</v>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:44:04.240706+00</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>P010</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>sess_1785759811750_03h7b21</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="2" t="n">
         <v>62075</v>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 12:45:07.396926+00</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>P011</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>sess_1785779493660_w2e74a9</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="2" t="n">
         <v>43520</v>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 17:53:09.563799+00</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>P011</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>sess_1785779493660_w2e74a9</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F33" s="3" t="n">
+      <c r="F33" s="2" t="n">
         <v>38025</v>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 17:53:46.926565+00</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>P011</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>sess_1785779493660_w2e74a9</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F34" s="3" t="n">
+      <c r="F34" s="2" t="n">
         <v>197819</v>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 17:57:05.406793+00</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>P012</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>sess_1785759393911_a3yx58l</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F35" s="3" t="n">
+      <c r="F35" s="2" t="n">
         <v>62651</v>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 17:59:38.561197+00</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>P012</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>sess_1785759393911_a3yx58l</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F36" s="3" t="n">
+      <c r="F36" s="2" t="n">
         <v>32732</v>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:00:10.168701+00</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>P012</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>sess_1785759393911_a3yx58l</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F37" s="3" t="n">
+      <c r="F37" s="2" t="n">
         <v>152897</v>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:02:44.324872+00</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>P013</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>sess_1785780300002_y11wqe9</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F38" s="3" t="n">
+      <c r="F38" s="2" t="n">
         <v>63229</v>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:07:28.202425+00</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>P013</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>sess_1785780300002_y11wqe9</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F39" s="3" t="n">
+      <c r="F39" s="2" t="n">
         <v>10373</v>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:07:38.508593+00</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>P013</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>sess_1785780300002_y11wqe9</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F40" s="3" t="n">
+      <c r="F40" s="2" t="n">
         <v>173998</v>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:10:33.789023+00</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>P014</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>sess_1785781818383_tdsj5ro</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F41" s="3" t="n">
+      <c r="F41" s="2" t="n">
         <v>93318</v>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:34:23.175337+00</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>P014</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>sess_1785781818383_tdsj5ro</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F42" s="3" t="n">
+      <c r="F42" s="2" t="n">
         <v>92920</v>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:35:56.578564+00</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>P014</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>sess_1785781818383_tdsj5ro</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F43" s="3" t="n">
+      <c r="F43" s="2" t="n">
         <v>71654</v>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 18:37:09.074846+00</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>P015</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>sess_1785784025815_9ywosu6</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F44" s="3" t="n">
+      <c r="F44" s="2" t="n">
         <v>12832</v>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:07:35.975807+00</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>P015</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>sess_1785784025815_9ywosu6</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F45" s="3" t="n">
+      <c r="F45" s="2" t="n">
         <v>10599</v>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:07:46.920501+00</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>P015</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>sess_1785784025815_9ywosu6</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F46" s="3" t="n">
+      <c r="F46" s="2" t="n">
         <v>81021</v>
       </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 19:09:08.684973+00</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>P016</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>sess_1785765159025_docr25l</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F47" s="3" t="n">
+      <c r="F47" s="2" t="n">
         <v>2807</v>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:53:21.726448+00</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>P016</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>sess_1785765159025_docr25l</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F48" s="3" t="n">
+      <c r="F48" s="2" t="n">
         <v>1630</v>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:53:23.329069+00</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>P016</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>sess_1785765159025_docr25l</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n">
+      <c r="F49" s="2" t="n">
         <v>38449</v>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:54:03.007891+00</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>P017</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>sess_1785765427281_9uxb322</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F50" s="3" t="n">
+      <c r="F50" s="2" t="n">
         <v>2516</v>
       </c>
-      <c r="G50" s="3" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:57:44.37177+00</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>P017</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>sess_1785765427281_9uxb322</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F51" s="3" t="n">
+      <c r="F51" s="2" t="n">
         <v>1820</v>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:57:46.045961+00</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>P017</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>sess_1785765427281_9uxb322</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F52" s="3" t="n">
+      <c r="F52" s="2" t="n">
         <v>48334</v>
       </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:58:35.960959+00</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>P018</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>sess_1785765545238_a11opnj</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F53" s="3" t="n">
+      <c r="F53" s="2" t="n">
         <v>2658</v>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:59:33.738035+00</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>P018</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>sess_1785765545238_a11opnj</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F54" s="3" t="n">
+      <c r="F54" s="2" t="n">
         <v>1714</v>
       </c>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 13:59:35.437098+00</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>P018</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>sess_1785765545238_a11opnj</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F55" s="3" t="n">
+      <c r="F55" s="2" t="n">
         <v>48594</v>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 14:00:25.373156+00</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>P019</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>sess_1785765645237_xxd26yy</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F56" s="3" t="n">
+      <c r="F56" s="2" t="n">
         <v>2264</v>
       </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 14:01:06.513331+00</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>P019</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>sess_1785765645237_xxd26yy</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F57" s="3" t="n">
+      <c r="F57" s="2" t="n">
         <v>2237</v>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 14:01:08.711986+00</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>P019</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>sess_1785765645237_xxd26yy</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F58" s="3" t="n">
+      <c r="F58" s="2" t="n">
         <v>34017</v>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 14:01:43.941897+00</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>P020</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>sess_1785765718963_66c0jpg</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>locate_product</t>
         </is>
       </c>
-      <c r="F59" s="3" t="n">
+      <c r="F59" s="2" t="n">
         <v>2263</v>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 14:02:50.889537+00</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>P020</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>sess_1785765718963_66c0jpg</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>add_to_basket</t>
         </is>
       </c>
-      <c r="F60" s="3" t="n">
+      <c r="F60" s="2" t="n">
         <v>1736</v>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 14:02:52.69649+00</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>P020</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>sess_1785765718963_66c0jpg</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>complete_checkout</t>
         </is>
       </c>
-      <c r="F61" s="3" t="n">
+      <c r="F61" s="2" t="n">
         <v>39066</v>
       </c>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>2026-08-03 14:03:33.208707+00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3587,17 +3647,17 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3658,163 +3718,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="2" t="n">
         <v>12434.2</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="2" t="n">
         <v>5096.6</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="2" t="n">
         <v>89037.39999999999</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="2" t="n">
         <v>106568.2</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="2" t="n">
         <v>12.43</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="I2" s="2" t="n">
         <v>5.1</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="J2" s="2" t="n">
         <v>89.04000000000001</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="K2" s="2" t="n">
         <v>106.57</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>18-25</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>18-25</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="2" t="n">
         <v>2501.6</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="2" t="n">
         <v>1827.4</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="2" t="n">
         <v>41692</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="2" t="n">
         <v>46021</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="2" t="n">
         <v>2.5</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="I3" s="2" t="n">
         <v>1.83</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="J3" s="2" t="n">
         <v>41.69</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="K3" s="2" t="n">
         <v>46.02</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="2" t="n">
         <v>55110</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="2" t="n">
         <v>36929.8</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>135477.8</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="2" t="n">
         <v>227517.6</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="2" t="n">
         <v>55.11</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="I4" s="2" t="n">
         <v>36.93</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="2" t="n">
         <v>135.48</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="K4" s="2" t="n">
         <v>227.52</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>65+</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="2" t="n">
         <v>7619.4</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="2" t="n">
         <v>4699.2</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="2" t="n">
         <v>80682.8</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="2" t="n">
         <v>93001.39999999999</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="2" t="n">
         <v>7.62</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="2" t="n">
         <v>4.7</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="J5" s="2" t="n">
         <v>80.68000000000001</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="K5" s="2" t="n">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3828,8 +3887,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3845,43 +3904,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>P01 / P02 / P98 / P99</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Incomplete or manual checks</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>P01, P02, P98, P99</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Incomplete or pilot/check rows</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>anonymous / verify_</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Junk / non-participant rows</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>anonymous / verify_ rows</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Not valid participant records</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>P008 extra rows</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Duplicate run removed; first complete set kept</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>P008 duplicate task set</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Second repeated run removed; first complete set kept</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3895,20 +3953,20 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>preparation_log</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P008/A: had 6 rows; kept first complete set of 3</t>
+          <t>P008 (A): duplicate task rows found; first complete set kept</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add dissertation statistical analysis workbook
Includes descriptives, Welch t-tests, Cohen's d, performance-gap
tables, and chart-ready summaries from the cleaned participant data.

Co-authored-by: David Olapade <David-O747@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exports/QuickBite_study_data_CLEAN.xlsx
+++ b/exports/QuickBite_study_data_CLEAN.xlsx
@@ -8,11 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="participant_summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="task_rows_clean" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="group_averages" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="excluded" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="prep_log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="dissertation_analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="participant_summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="task_rows_clean" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="group_averages" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="excluded" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="prep_log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="descriptives_seconds" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ttests" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="cohens_d" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="performance_gap_A" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +39,20 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,8 +64,13 @@
         <fgColor rgb="00333333"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -70,14 +92,35 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,9 +499,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -473,9 +514,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -511,9 +550,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -528,9 +565,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -559,9 +594,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -597,9 +630,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -619,6 +650,830 @@
         <is>
           <t>so they share a session_id. Later sessions used separate browser sessions.</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Comparison family</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Group 2</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Cohen's d</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>|d|</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>5.099</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>5.099</v>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>3.958</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>3.958</v>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>2.618</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>2.618</v>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>3.435</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>3.435</v>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>2.254</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2.254</v>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>1.348</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>1.348</v>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>2.571</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>2.571</v>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>-1.334</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>1.334</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>-1.067</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1.067</v>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>-2.311</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2.311</v>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>-2.117</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>2.117</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>-1.764</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1.764</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>-2.165</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2.165</v>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>-2.671</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>2.671</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Positive d means Group 1 mean &gt; Group 2 mean (Group 1 slower in ms)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Site version</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Younger mean (s)</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Older mean (s)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Gap older-younger (s)</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Older slower by %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>55.11</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>42.68</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>343.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>31.83</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>624.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>89.04000000000001</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>135.48</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>46.44</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>52.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>106.57</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>227.52</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>120.95</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>113.5</v>
       </c>
     </row>
   </sheetData>
@@ -627,6 +1482,158 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>DISSERTATION ANALYSIS SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>See QuickBite_dissertation_analysis.xlsx for full write-up sheets, significance highlighting, and embedded figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>This workbook now also contains descriptives_seconds, ttests, cohens_d, and performance_gap_A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Mean completion times (seconds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Younger / Version A</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>89.04000000000001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>106.57</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Younger / Version B</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="D9" t="n">
+        <v>41.69</v>
+      </c>
+      <c r="E9" t="n">
+        <v>46.02</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Older / Version A</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>55.11</v>
+      </c>
+      <c r="C10" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="D10" t="n">
+        <v>135.48</v>
+      </c>
+      <c r="E10" t="n">
+        <v>227.52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Older / Version B</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="E11" t="n">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1478,7 +2485,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3638,7 +4645,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3878,7 +4885,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3944,7 +4951,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3973,4 +4980,1218 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Locate product M</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Locate product Mdn</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Locate product SD</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Add to basket M</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Add to basket Mdn</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Add to basket SD</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Complete checkout M</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Complete checkout Mdn</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Complete checkout SD</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Total completion M</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Total completion Mdn</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Total completion SD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Younger / Version A</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>12.64</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>89.04000000000001</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>86.12</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>106.57</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N2" s="7" t="n">
+        <v>24.08</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Younger / Version B</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>41.69</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>39.07</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>46.02</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>43.06</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>6.47</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Older / Version A</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>55.11</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>62.65</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>32.73</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>33.74</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>135.48</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>152.9</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>227.52</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>248.28</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>69.98</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Older / Version B</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>69.42</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>24.63</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>80.23999999999999</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>24.02</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Comparison family</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Group 2</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>n1</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>n2</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Mean 1 (s)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Mean 2 (s)</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>df</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Significant (p&lt;.05)</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>8.061999999999999</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="L2" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A slower than 18-25 B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>6.258</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A slower than 18-25 B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>89.04000000000001</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>41.69</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>4.139</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A slower than 18-25 B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Younger: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>106.57</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>46.02</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>5.431</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A slower than 18-25 B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>55.11</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>3.564</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>65+ A slower than 65+ B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>2.131</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>0.0994</v>
+      </c>
+      <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>65+ A slower than 65+ B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>135.48</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>1.992</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0.09810000000000001</v>
+      </c>
+      <c r="L8" s="7" t="inlineStr"/>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>65+ A slower than 65+ B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Older: Version A vs Version B</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>227.52</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>4.065</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>65+ A slower than 65+ B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>55.11</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>-3.21</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>0.0318</v>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A faster than 65+ A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>-2.109</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>0.1025</v>
+      </c>
+      <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A faster than 65+ A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>89.04000000000001</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>135.48</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>-1.687</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>0.1473</v>
+      </c>
+      <c r="L12" s="7" t="inlineStr"/>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A faster than 65+ A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Version A: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>65+ A</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>106.57</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>227.52</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>-3.654</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>18-25 A faster than 65+ A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Locate product</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>-3.347</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>0.0282</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B faster than 65+ B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Add to basket</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>-2.789</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>0.0482</v>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B faster than 65+ B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Complete checkout</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>41.69</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>-3.424</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B faster than 65+ B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Version B: Younger vs Older</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Total completion</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>65+ B</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>46.02</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>-4.224</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>0.0101</v>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>18-25 B faster than 65+ B</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>